<commit_message>
Connected the Multinomial Logit with the backend
</commit_message>
<xml_diff>
--- a/MILP/model_output/TS_Subproblem_Solution.xlsx
+++ b/MILP/model_output/TS_Subproblem_Solution.xlsx
@@ -532,7 +532,7 @@
         <v>24</v>
       </c>
       <c r="G2">
-        <v>55.44000000000007</v>
+        <v>55.44000000000008</v>
       </c>
       <c r="H2">
         <v>221</v>
@@ -590,7 +590,7 @@
         <v>25</v>
       </c>
       <c r="G4">
-        <v>55.44000000000007</v>
+        <v>55.44000000000008</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>26</v>
       </c>
       <c r="G5">
-        <v>55.44000000000007</v>
+        <v>55.44000000000008</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -727,16 +727,16 @@
         <v>35</v>
       </c>
       <c r="C2">
-        <v>55.44000000000007</v>
+        <v>55.44000000000008</v>
       </c>
       <c r="D2">
-        <v>55.44000000000007</v>
+        <v>55.44000000000008</v>
       </c>
       <c r="E2">
-        <v>55.43999999999998</v>
+        <v>55.44000000000008</v>
       </c>
       <c r="F2">
-        <v>100.0000000000002</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
         <v>27</v>
@@ -756,10 +756,10 @@
         <v>55.44000000000007</v>
       </c>
       <c r="E3">
-        <v>55.4399999999999</v>
+        <v>55.4399999999994</v>
       </c>
       <c r="F3">
-        <v>100.0000000000003</v>
+        <v>100.0000000000012</v>
       </c>
       <c r="G3" t="s">
         <v>28</v>

</xml_diff>